<commit_message>
Shared my feelings and buddy
</commit_message>
<xml_diff>
--- a/12614271.xlsx
+++ b/12614271.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Sem 1 MCA\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E93A50A3-A81E-44A2-9426-B359A99E1386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D816758-6F3A-406A-BD9A-752A72D78471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="74">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -230,6 +230,24 @@
   </si>
   <si>
     <t>Studied in Library</t>
+  </si>
+  <si>
+    <t>Not great</t>
+  </si>
+  <si>
+    <t>Decent</t>
+  </si>
+  <si>
+    <t>Bad</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Missed my partner.</t>
+  </si>
+  <si>
+    <t>It was fine till evening,  then I got told  something things from my partner.</t>
   </si>
 </sst>
 </file>
@@ -1240,53 +1258,97 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>46284</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="str">
+      <c r="B11" s="14">
+        <v>360</v>
+      </c>
+      <c r="C11" s="14">
+        <v>50</v>
+      </c>
+      <c r="D11" s="14">
+        <v>200</v>
+      </c>
+      <c r="E11" s="14">
+        <v>0</v>
+      </c>
+      <c r="F11" s="14">
+        <v>90</v>
+      </c>
+      <c r="G11" s="14">
+        <v>2</v>
+      </c>
+      <c r="H11" s="14">
+        <v>60</v>
+      </c>
+      <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
+        <v>760</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="17"/>
+        <v>680</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>46285</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+      <c r="B12" s="14">
+        <v>480</v>
+      </c>
+      <c r="C12" s="14">
+        <v>20</v>
+      </c>
+      <c r="D12" s="14">
+        <v>150</v>
+      </c>
+      <c r="E12" s="14">
+        <v>10</v>
+      </c>
+      <c r="F12" s="14">
+        <v>0</v>
+      </c>
+      <c r="G12" s="14">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14">
+        <v>60</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>720</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
+        <v>720</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
@@ -9868,7 +9930,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations disablePrompts="1" count="3">
     <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6:K401" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Excellent,Good,Neutral,Low,Stressed"</formula1>
       <formula2>0</formula2>

</xml_diff>

<commit_message>
DOne for today !
</commit_message>
<xml_diff>
--- a/12614271.xlsx
+++ b/12614271.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Sem 1 MCA\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D816758-6F3A-406A-BD9A-752A72D78471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2FEF44D-DAD2-4E37-9114-37C4B9C92C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="78">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -249,6 +249,18 @@
   <si>
     <t>It was fine till evening,  then I got told  something things from my partner.</t>
   </si>
+  <si>
+    <t>8.5/10</t>
+  </si>
+  <si>
+    <t>4.5/10</t>
+  </si>
+  <si>
+    <t>Got it in evening</t>
+  </si>
+  <si>
+    <t>Got to study for RPL</t>
+  </si>
 </sst>
 </file>
 
@@ -386,7 +398,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -430,6 +442,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1354,49 +1369,93 @@
       <c r="A13" s="8">
         <v>46286</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+      <c r="B13" s="14">
+        <v>330</v>
+      </c>
+      <c r="C13" s="14">
+        <v>30</v>
+      </c>
+      <c r="D13" s="14">
+        <v>180</v>
+      </c>
+      <c r="E13" s="14">
+        <v>20</v>
+      </c>
+      <c r="F13" s="14">
+        <v>400</v>
+      </c>
+      <c r="G13" s="14">
+        <v>7</v>
+      </c>
+      <c r="H13" s="14">
+        <v>40</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>1000</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
+        <v>440</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>46287</v>
       </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="B14" s="14">
+        <v>300</v>
+      </c>
+      <c r="C14" s="14">
+        <v>20</v>
+      </c>
+      <c r="D14" s="14">
+        <v>160</v>
+      </c>
+      <c r="E14" s="14">
+        <v>20</v>
+      </c>
+      <c r="F14" s="14">
+        <v>310</v>
+      </c>
+      <c r="G14" s="14">
+        <v>5</v>
+      </c>
+      <c r="H14" s="14">
+        <v>50</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>860</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
+        <v>580</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L14" s="21">
+        <v>46302</v>
+      </c>
+      <c r="M14" s="21">
+        <v>46300</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
@@ -9930,7 +9989,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="3">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6:K401" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Excellent,Good,Neutral,Low,Stressed"</formula1>
       <formula2>0</formula2>

</xml_diff>